<commit_message>
Finieshed with the second revision of List of Contracts report - prettyfied and excluded delta cashflow calculation
</commit_message>
<xml_diff>
--- a/src/main/resources/ru/stnovator/finassist/report/list-of-contracts.xlsx
+++ b/src/main/resources/ru/stnovator/finassist/report/list-of-contracts.xlsx
@@ -13,21 +13,21 @@
   <definedNames>
     <definedName function="false" hidden="false" name="Header" vbProcedure="false">Sheet1!$A$1:$G$2</definedName>
     <definedName function="false" hidden="false" name="Customer" vbProcedure="false">Sheet1!$A$3:$G$3</definedName>
-    <definedName function="false" hidden="false" name="Contract" vbProcedure="false">Sheet1!$A$4:$E$5</definedName>
-    <definedName function="false" hidden="false" name="Project" vbProcedure="false">Sheet1!$A$6:$D$6</definedName>
-    <definedName function="false" hidden="false" name="ProjectCashflowHeader" vbProcedure="false">Sheet1!$A$7:$D$7</definedName>
-    <definedName function="false" hidden="false" name="ProjectCashflowRecord" vbProcedure="false">Sheet1!$A$8:$D$8</definedName>
-    <definedName function="false" hidden="false" name="ProjectCashflowTotal" vbProcedure="false">Sheet1!$A$9:$D$9</definedName>
-    <definedName function="false" hidden="false" name="ProjectSpacer" vbProcedure="false">Sheet1!$A$10:$G$10</definedName>
-    <definedName function="false" hidden="false" name="ContractSpacer" vbProcedure="false">Sheet1!$A$11:$G$11</definedName>
-    <definedName function="false" hidden="false" name="CustomerSpacer" vbProcedure="false">Sheet1!$A$12:$G$13</definedName>
+    <definedName function="false" hidden="false" name="Contract" vbProcedure="false">Sheet1!$A$4:$G$6</definedName>
+    <definedName function="false" hidden="false" name="Project" vbProcedure="false">Sheet1!$A$7:$G$7</definedName>
+    <definedName function="false" hidden="false" name="ProjectCashflowHeader" vbProcedure="false">Sheet1!$A$8:$C$8</definedName>
+    <definedName function="false" hidden="false" name="ProjectCashflowRecord" vbProcedure="false">Sheet1!$A$9:$C$9</definedName>
+    <definedName function="false" hidden="false" name="ProjectCashflowTotal" vbProcedure="false">Sheet1!$A$10:$C$10</definedName>
+    <definedName function="false" hidden="false" name="ProjectSpacer" vbProcedure="false">Sheet1!$A$11:$G$11</definedName>
+    <definedName function="false" hidden="false" name="ContractSpacer" vbProcedure="false">Sheet1!$A$12:$G$12</definedName>
+    <definedName function="false" hidden="false" name="CustomerSpacer" vbProcedure="false">Sheet1!$A$13:$G$14</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">Список контрактов</t>
   </si>
@@ -89,9 +89,6 @@
     <t xml:space="preserve">Плановая сумма оплаты</t>
   </si>
   <si>
-    <t xml:space="preserve">Дельта</t>
-  </si>
-  <si>
     <t xml:space="preserve">${cashflowDate}</t>
   </si>
   <si>
@@ -101,9 +98,6 @@
     <t xml:space="preserve">${paymentSum}</t>
   </si>
   <si>
-    <t xml:space="preserve">${deltaSum}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Итого:</t>
   </si>
   <si>
@@ -113,56 +107,77 @@
     <t xml:space="preserve">${paymentTotal}</t>
   </si>
   <si>
-    <t xml:space="preserve">${finalDelta}</t>
+    <t xml:space="preserve">Дата отчета:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${reportDate}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${addendumInfoLabel}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${addendumNumber}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${addendumDateLabel}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${addendumEffectiveDate}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
   <fonts count="6">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF111827"/>
       <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF0F172A"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,143 +186,122 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.05"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5B7FA3"/>
+        <bgColor rgb="FF5B7FA3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF1FB"/>
+        <bgColor rgb="FFEAF1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD8E4F2"/>
+        <bgColor rgb="FFD8E4F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+  <borders count="4">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB8C4D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB8C4D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB8C4D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB8C4D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF5B7FA3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF5B7FA3"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF5B7FA3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF5B7FA3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7C8EA3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7C8EA3"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF44546A"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF44546A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF2F2F2"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -488,19 +482,19 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="10.39453125" defaultRowHeight="16" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="18" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col min="1" max="1" width="26" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="2" max="2" width="24" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="3" max="3" width="20" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="4" max="4" width="20" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="5" max="5" width="20" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="6" max="6" width="20" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="7" max="7" width="18" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="28" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -511,112 +505,179 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="22" customHeight="true">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+    </row>
+    <row r="3" ht="30" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" ht="24" customHeight="true">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+    </row>
+    <row r="5" ht="30" customHeight="true">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="6" ht="22" customHeight="true">
       <c r="A6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" ht="38" customHeight="true">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" ht="40" customHeight="true">
+      <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="s">
+    </row>
+    <row r="9" ht="22" customHeight="true">
+      <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="6" t="s">
+    </row>
+    <row r="10" ht="24" customHeight="true">
+      <c r="A10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="B10" s="9" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="C10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    </row>
+    <row r="11" ht="10" customHeight="true">
+      <c r="A11"/>
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
+    </row>
+    <row r="12" ht="10" customHeight="true">
+      <c r="A12"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+    </row>
+    <row r="13" ht="10" customHeight="true">
+      <c r="A13"/>
+      <c r="B13"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
+    </row>
+    <row r="14" ht="10" customHeight="true">
+      <c r="A14"/>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="F7:G7"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>